<commit_message>
Seb ruling: 2+-more-goals markets DROPPED from product entirely (calculator + per-second CSV). Overshoot gate stays as model-health diagnostic only
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012si27ZfLSnpNPfN3rGmhCN
</commit_message>
<xml_diff>
--- a/live_model/3mapgot_calculator_v2.xlsx
+++ b/live_model/3mapgot_calculator_v2.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="813">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2109" uniqueCount="811">
   <si>
     <t xml:space="preserve">3MAPGOT CALCULATOR v2.3 — per-second 10%-EV lines (built from dense MC grid, n=30k, seed 7)</t>
   </si>
@@ -64,7 +64,7 @@
     <t xml:space="preserve">- Leader market: model runs ~5pts LOW (under investigation). Overs ONLY — never bet leader-market unders off this sheet.</t>
   </si>
   <si>
-    <t xml:space="preserve">- WITHDRAWN: 2+ more goals while net is ALREADY empty. Model overshoots that corner; do not bet it (docs/WITHDRAWN_MARKETS.md).</t>
+    <t xml:space="preserve">- DROPPED (Seb 2026-07-25): all 2+-more-goals markets. Not part of the product.</t>
   </si>
   <si>
     <t xml:space="preserve">- Low-tail coaches (Huska, Tortorella, McLellan): home/fav context multipliers do NOT apply — enter 'n'/'even' for them.</t>
@@ -2272,9 +2272,6 @@
     <t xml:space="preserve">P(any more goal) — game total over</t>
   </si>
   <si>
-    <t xml:space="preserve">P(2+ more goals) — WITHDRAWN if pulled</t>
-  </si>
-  <si>
     <t xml:space="preserve">P(LEADER scores again) — team total over (model ~5pts LOW; Overs only)</t>
   </si>
   <si>
@@ -2288,9 +2285,6 @@
   </si>
   <si>
     <t xml:space="preserve">P(any more goal)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P(2+ more goals)</t>
   </si>
   <si>
     <t xml:space="preserve">P(LEADER scores again)</t>
@@ -24273,7 +24267,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -24431,11 +24425,11 @@
       </c>
       <c r="D16" s="5" t="n">
         <f aca="false">(1-$F$11)*((1-$F$10)*B23+$F$10*C23)+$F$11*((1-$F$10)*D23+$F$10*E23)</f>
-        <v>0.3514</v>
+        <v>0.6227</v>
       </c>
       <c r="E16" s="1" t="str">
         <f aca="false">IF(D16&lt;=0,"n/a",IF((1+$D$8-D16)/D16&gt;=1,"+"&amp;TEXT(ROUND((1+$D$8-D16)/D16*100,0),"0"),"-"&amp;TEXT(ROUND(100/((1+$D$8-D16)/D16),0),"0")))</f>
-        <v>+213</v>
+        <v>-130</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24444,47 +24438,30 @@
       </c>
       <c r="D17" s="5" t="n">
         <f aca="false">(1-$F$11)*((1-$F$10)*B24+$F$10*C24)+$F$11*((1-$F$10)*D24+$F$10*E24)</f>
-        <v>0.6227</v>
+        <v>0.4404</v>
       </c>
       <c r="E17" s="1" t="str">
         <f aca="false">IF(D17&lt;=0,"n/a",IF((1+$D$8-D17)/D17&gt;=1,"+"&amp;TEXT(ROUND((1+$D$8-D17)/D17*100,0),"0"),"-"&amp;TEXT(ROUND(100/((1+$D$8-D17)/D17),0),"0")))</f>
-        <v>-130</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>751</v>
-      </c>
-      <c r="D18" s="5" t="n">
-        <f aca="false">(1-$F$11)*((1-$F$10)*B25+$F$10*C25)+$F$11*((1-$F$10)*D25+$F$10*E25)</f>
-        <v>0.4404</v>
-      </c>
-      <c r="E18" s="1" t="str">
-        <f aca="false">IF(D18&lt;=0,"n/a",IF((1+$D$8-D18)/D18&gt;=1,"+"&amp;TEXT(ROUND((1+$D$8-D18)/D18*100,0),"0"),"-"&amp;TEXT(ROUND(100/((1+$D$8-D18)/D18),0),"0")))</f>
         <v>+150</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="D19" s="6" t="str">
         <f aca="false">IF(AND(D4="pulled",D9&gt;420),"EXTRAPOLATED — no real pulls this early","ok")</f>
         <v>ok</v>
       </c>
-      <c r="E19" s="6" t="str">
-        <f aca="false">IF(D4="pulled","2+ goals market WITHDRAWN in pulled state — do not bet","")</f>
-        <v/>
-      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">INDEX(PRICES!F:F,MATCH($B$12,PRICES!A:A,0))</f>
@@ -24505,63 +24482,42 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="B23" s="7" t="n">
-        <f aca="false">INDEX(PRICES!G:G,MATCH($B$12,PRICES!A:A,0))</f>
-        <v>0.3365</v>
+        <f aca="false">INDEX(PRICES!H:H,MATCH($B$12,PRICES!A:A,0))</f>
+        <v>0.5915</v>
       </c>
       <c r="C23" s="7" t="n">
-        <f aca="false">INDEX(PRICES!G:G,MATCH($C$12,PRICES!A:A,0))</f>
-        <v>0.3514</v>
+        <f aca="false">INDEX(PRICES!H:H,MATCH($C$12,PRICES!A:A,0))</f>
+        <v>0.6227</v>
       </c>
       <c r="D23" s="7" t="n">
-        <f aca="false">INDEX(PRICES!G:G,MATCH($D$12,PRICES!A:A,0))</f>
-        <v>0.3453</v>
+        <f aca="false">INDEX(PRICES!H:H,MATCH($D$12,PRICES!A:A,0))</f>
+        <v>0.5998</v>
       </c>
       <c r="E23" s="7" t="n">
-        <f aca="false">INDEX(PRICES!G:G,MATCH($E$12,PRICES!A:A,0))</f>
-        <v>0.3595</v>
+        <f aca="false">INDEX(PRICES!H:H,MATCH($E$12,PRICES!A:A,0))</f>
+        <v>0.6294</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B24" s="7" t="n">
-        <f aca="false">INDEX(PRICES!H:H,MATCH($B$12,PRICES!A:A,0))</f>
-        <v>0.5915</v>
-      </c>
-      <c r="C24" s="7" t="n">
-        <f aca="false">INDEX(PRICES!H:H,MATCH($C$12,PRICES!A:A,0))</f>
-        <v>0.6227</v>
-      </c>
-      <c r="D24" s="7" t="n">
-        <f aca="false">INDEX(PRICES!H:H,MATCH($D$12,PRICES!A:A,0))</f>
-        <v>0.5998</v>
-      </c>
-      <c r="E24" s="7" t="n">
-        <f aca="false">INDEX(PRICES!H:H,MATCH($E$12,PRICES!A:A,0))</f>
-        <v>0.6294</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>757</v>
-      </c>
-      <c r="B25" s="7" t="n">
         <f aca="false">INDEX(PRICES!I:I,MATCH($B$12,PRICES!A:A,0))</f>
         <v>0.4139</v>
       </c>
-      <c r="C25" s="7" t="n">
+      <c r="C24" s="7" t="n">
         <f aca="false">INDEX(PRICES!I:I,MATCH($C$12,PRICES!A:A,0))</f>
         <v>0.4404</v>
       </c>
-      <c r="D25" s="7" t="n">
+      <c r="D24" s="7" t="n">
         <f aca="false">INDEX(PRICES!I:I,MATCH($D$12,PRICES!A:A,0))</f>
         <v>0.4185</v>
       </c>
-      <c r="E25" s="7" t="n">
+      <c r="E24" s="7" t="n">
         <f aca="false">INDEX(PRICES!I:I,MATCH($E$12,PRICES!A:A,0))</f>
         <v>0.4428</v>
       </c>
@@ -24591,30 +24547,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>756</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>757</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>758</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>759</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>760</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>761</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>762</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>763</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>764</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>9</v>
@@ -24635,7 +24591,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>8</v>
@@ -24656,7 +24612,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>5</v>
@@ -24677,7 +24633,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>12</v>
@@ -24698,7 +24654,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>15</v>
@@ -24719,7 +24675,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>3</v>
@@ -24740,7 +24696,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>5</v>
@@ -24761,7 +24717,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>11</v>
@@ -24782,7 +24738,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>1</v>
@@ -24800,12 +24756,12 @@
         <v>2</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>7</v>
@@ -24826,7 +24782,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>7</v>
@@ -24847,7 +24803,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>11</v>
@@ -24868,7 +24824,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>3</v>
@@ -24889,7 +24845,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>9</v>
@@ -24910,7 +24866,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>6</v>
@@ -24931,7 +24887,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>7</v>
@@ -24952,7 +24908,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>3</v>
@@ -24973,7 +24929,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>3</v>
@@ -24994,7 +24950,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>7</v>
@@ -25015,7 +24971,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>6</v>
@@ -25036,7 +24992,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>8</v>
@@ -25057,7 +25013,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>6</v>
@@ -25078,7 +25034,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>6</v>
@@ -25099,7 +25055,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>5</v>
@@ -25120,7 +25076,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>0</v>
@@ -25138,12 +25094,12 @@
         <v>4</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>0</v>
@@ -25164,7 +25120,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>4</v>
@@ -25185,7 +25141,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>1</v>
@@ -25206,7 +25162,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>7</v>
@@ -25227,7 +25183,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>8</v>
@@ -25248,7 +25204,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>0</v>
@@ -25266,12 +25222,12 @@
         <v>1</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>4</v>
@@ -25292,7 +25248,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>4</v>
@@ -25313,7 +25269,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>4</v>
@@ -25334,7 +25290,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>5</v>
@@ -25355,7 +25311,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>1</v>
@@ -25376,7 +25332,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>3</v>
@@ -25397,7 +25353,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>0</v>
@@ -25418,7 +25374,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>2</v>
@@ -25439,7 +25395,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>2</v>
@@ -25460,7 +25416,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>2</v>
@@ -25478,12 +25434,12 @@
         <v>36</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>4</v>
@@ -25504,7 +25460,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>2</v>
@@ -25522,12 +25478,12 @@
         <v>27</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>1</v>
@@ -25545,12 +25501,12 @@
         <v>41</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>0</v>
@@ -25571,7 +25527,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Timing de-noised (Seb: averages are opportunity-gated): 4-season persistence refit 0.608 (up from 0.375), shifts attenuated + n-shrunk in TEAM LINES; opportunity caveat in docs; softened past-his-time guidance
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012si27ZfLSnpNPfN3rGmhCN
</commit_message>
<xml_diff>
--- a/live_model/3mapgot_calculator_v2.xlsx
+++ b/live_model/3mapgot_calculator_v2.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3433" uniqueCount="2124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3434" uniqueCount="2125">
   <si>
     <t xml:space="preserve">3MAPGOT CALCULATOR v2.3 — per-second 10%-EV lines (built from dense MC grid, n=30k, seed 7)</t>
   </si>
@@ -6219,10 +6219,13 @@
     <t xml:space="preserve">Leader -3.5 (wins by 4+)</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes: timing snapped to nearest grid step (max 30s, ~1pt effect). 100%% pullers: use 0.99.</t>
+    <t xml:space="preserve">Notes: timing snapped to nearest grid step (max 30s, ~1pt effect). 100% pullers: use 0.99.</t>
   </si>
   <si>
     <t xml:space="preserve">5v5 only — PP/pulled states not bettable (Seb rulings).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Timing input: observed averages are opportunity-noise — if your read is from &lt;10 pulls, enter something between his avg and 4:19.</t>
   </si>
   <si>
     <t xml:space="preserve">Game total OVER</t>
@@ -58482,9 +58485,14 @@
         <v>2065</v>
       </c>
     </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>2066</v>
+      </c>
+    </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>2066</v>
+        <v>2067</v>
       </c>
       <c r="B21" s="7" t="n">
         <f aca="false">INDEX(MANUAL_PRICES!E:E,MATCH($B$11,MANUAL_PRICES!A:A,0))</f>
@@ -58505,7 +58513,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>2067</v>
+        <v>2068</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">INDEX(MANUAL_PRICES!F:F,MATCH($B$11,MANUAL_PRICES!A:A,0))</f>
@@ -58526,7 +58534,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>2068</v>
+        <v>2069</v>
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">INDEX(MANUAL_PRICES!G:G,MATCH($B$11,MANUAL_PRICES!A:A,0))</f>
@@ -58570,30 +58578,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>2069</v>
+        <v>2070</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2070</v>
+        <v>2071</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2071</v>
+        <v>2072</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2072</v>
+        <v>2073</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>2073</v>
+        <v>2074</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>2074</v>
+        <v>2075</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>2075</v>
+        <v>2076</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>2076</v>
+        <v>2077</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>9</v>
@@ -58614,7 +58622,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>2077</v>
+        <v>2078</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>8</v>
@@ -58635,7 +58643,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>2078</v>
+        <v>2079</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>5</v>
@@ -58656,7 +58664,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>2079</v>
+        <v>2080</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>12</v>
@@ -58677,7 +58685,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>2080</v>
+        <v>2081</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>15</v>
@@ -58698,7 +58706,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>2081</v>
+        <v>2082</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>3</v>
@@ -58719,7 +58727,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>2082</v>
+        <v>2083</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>5</v>
@@ -58740,7 +58748,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>2083</v>
+        <v>2084</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>11</v>
@@ -58761,7 +58769,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>2084</v>
+        <v>2085</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>1</v>
@@ -58779,12 +58787,12 @@
         <v>2</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>2085</v>
+        <v>2086</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>2086</v>
+        <v>2087</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>7</v>
@@ -58805,7 +58813,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>2087</v>
+        <v>2088</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>7</v>
@@ -58826,7 +58834,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>2088</v>
+        <v>2089</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>11</v>
@@ -58847,7 +58855,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>2089</v>
+        <v>2090</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>3</v>
@@ -58868,7 +58876,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>9</v>
@@ -58889,7 +58897,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>2091</v>
+        <v>2092</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>6</v>
@@ -58910,7 +58918,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>2092</v>
+        <v>2093</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>7</v>
@@ -58931,7 +58939,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>2093</v>
+        <v>2094</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>3</v>
@@ -58952,7 +58960,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>2094</v>
+        <v>2095</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>3</v>
@@ -58973,7 +58981,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>2095</v>
+        <v>2096</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>7</v>
@@ -58994,7 +59002,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>2096</v>
+        <v>2097</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>6</v>
@@ -59015,7 +59023,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>2097</v>
+        <v>2098</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>8</v>
@@ -59036,7 +59044,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>2098</v>
+        <v>2099</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>6</v>
@@ -59057,7 +59065,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>2099</v>
+        <v>2100</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>6</v>
@@ -59078,7 +59086,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>2100</v>
+        <v>2101</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>5</v>
@@ -59099,7 +59107,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>2101</v>
+        <v>2102</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>0</v>
@@ -59117,12 +59125,12 @@
         <v>4</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>2085</v>
+        <v>2086</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>2102</v>
+        <v>2103</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>0</v>
@@ -59143,7 +59151,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>2103</v>
+        <v>2104</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>4</v>
@@ -59164,7 +59172,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>2104</v>
+        <v>2105</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>1</v>
@@ -59185,7 +59193,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>2105</v>
+        <v>2106</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>7</v>
@@ -59206,7 +59214,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>2106</v>
+        <v>2107</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>8</v>
@@ -59227,7 +59235,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>2107</v>
+        <v>2108</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>0</v>
@@ -59245,12 +59253,12 @@
         <v>1</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>2085</v>
+        <v>2086</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>2108</v>
+        <v>2109</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>4</v>
@@ -59271,7 +59279,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>2109</v>
+        <v>2110</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>4</v>
@@ -59292,7 +59300,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>2110</v>
+        <v>2111</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>4</v>
@@ -59313,7 +59321,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>2111</v>
+        <v>2112</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>5</v>
@@ -59334,7 +59342,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>2112</v>
+        <v>2113</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>1</v>
@@ -59355,7 +59363,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>2113</v>
+        <v>2114</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>3</v>
@@ -59376,7 +59384,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>2114</v>
+        <v>2115</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>0</v>
@@ -59397,7 +59405,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>2115</v>
+        <v>2116</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>2</v>
@@ -59418,7 +59426,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>2116</v>
+        <v>2117</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>2</v>
@@ -59439,7 +59447,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>2</v>
@@ -59457,12 +59465,12 @@
         <v>36</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>2118</v>
+        <v>2119</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>2119</v>
+        <v>2120</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>4</v>
@@ -59483,7 +59491,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>2120</v>
+        <v>2121</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>2</v>
@@ -59501,12 +59509,12 @@
         <v>27</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>2118</v>
+        <v>2119</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>2121</v>
+        <v>2122</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>1</v>
@@ -59524,12 +59532,12 @@
         <v>41</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>2118</v>
+        <v>2119</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>2122</v>
+        <v>2123</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>0</v>
@@ -59550,7 +59558,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>2123</v>
+        <v>2124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebuild calculator + lines workbooks on ruling-29 profiles
</commit_message>
<xml_diff>
--- a/live_model/3mapgot_calculator_v2.xlsx
+++ b/live_model/3mapgot_calculator_v2.xlsx
@@ -520,21 +520,21 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>- leader TT over: realized ROI +21.3%, CI [+7.3%, +35.9%] — PROVEN &gt;10%</t>
+          <t>- leader TT over: realized ROI +24.0%, CI [+9.6%, +39.0%] — PROVEN &gt;10%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>- game total over: realized ROI +9.3%, CI [-0.9%, +20.1%] — positive, 10% not proven</t>
+          <t>- game total over: realized ROI +11.2%, CI [+0.8%, +22.6%] — positive, 10% not proven</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>- leader -3.5: realized ROI +2.5%, CI [-13.8%, +19.3%] — CI includes 0: treat edges as optimistic</t>
+          <t>- leader -3.5: realized ROI +4.8%, CI [-11.8%, +22.6%] — CI includes 0: treat edges as optimistic</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuilt calculator + lines workbooks on rulings 29-30 coach numbers
</commit_message>
<xml_diff>
--- a/live_model/3mapgot_calculator_v2.xlsx
+++ b/live_model/3mapgot_calculator_v2.xlsx
@@ -520,21 +520,21 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>- leader TT over: realized ROI +24.0%, CI [+9.6%, +39.0%] — PROVEN &gt;10%</t>
+          <t>- leader TT over: realized ROI +23.9%, CI [+9.6%, +38.9%] — PROVEN &gt;10%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>- game total over: realized ROI +11.2%, CI [+0.8%, +22.6%] — positive, 10% not proven</t>
+          <t>- game total over: realized ROI +11.1%, CI [+0.7%, +22.5%] — positive, 10% not proven</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>- leader -3.5: realized ROI +4.8%, CI [-11.8%, +22.6%] — CI includes 0: treat edges as optimistic</t>
+          <t>- leader -3.5: realized ROI +4.7%, CI [-11.9%, +22.5%] — CI includes 0: treat edges as optimistic</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
workbooks rebuilt on ruling-32 numbers
</commit_message>
<xml_diff>
--- a/live_model/3mapgot_calculator_v2.xlsx
+++ b/live_model/3mapgot_calculator_v2.xlsx
@@ -520,21 +520,21 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>- leader TT over: realized ROI +23.9%, CI [+9.6%, +38.9%] — PROVEN &gt;10%</t>
+          <t>- leader TT over: realized ROI +24.6%, CI [+10.0%, +39.9%] — PROVEN &gt;10%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>- game total over: realized ROI +11.1%, CI [+0.7%, +22.5%] — positive, 10% not proven</t>
+          <t>- game total over: realized ROI +11.6%, CI [+1.0%, +23.0%] — positive, 10% not proven</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>- leader -3.5: realized ROI +4.7%, CI [-11.9%, +22.5%] — CI includes 0: treat edges as optimistic</t>
+          <t>- leader -3.5: realized ROI +5.6%, CI [-11.6%, +23.7%] — CI includes 0: treat edges as optimistic</t>
         </is>
       </c>
     </row>

</xml_diff>